<commit_message>
clean_data.py. drop_alternatives_with_wrong_values modifique eliminacion de outliers. Quite media y desvio. Ahora utilizo rango intercaurtil.
pagina_web.py. Agregue chart y expander.
</commit_message>
<xml_diff>
--- a/data/data_preparation/celulares/df_cust_needs.xlsx
+++ b/data/data_preparation/celulares/df_cust_needs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,94 +486,58 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>señal</t>
+          <t>pantalla</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tiene buena señal</t>
+          <t>buena calidad pantalla</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>pantalla</t>
+          <t>usar</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>buen tamaño pantalla</t>
+          <t>super facil usar</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>huella</t>
+          <t>diseño</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>desbloqueo huella digital</t>
+          <t>celular buen diseño</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>juegos</t>
+          <t>velocidad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>corre bien juegos</t>
+          <t>buena velocidad procesamiento</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>sistema</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
-        <is>
-          <t>sistema operativo bueno</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>diseño</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>celular buen diseño</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>procesador</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>tiene buen procesador</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>marca</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
         <is>
           <t>mejor marca celulares</t>
         </is>

</xml_diff>

<commit_message>
Mejora de notas Eliminacion de funciones en desuso
</commit_message>
<xml_diff>
--- a/data/data_preparation/celulares/df_cust_needs.xlsx
+++ b/data/data_preparation/celulares/df_cust_needs.xlsx
@@ -1,112 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10520"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A229E385-99DA-FC46-AB55-861BC5428573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
-  <si>
-    <t>cust_needs_three_words</t>
-  </si>
-  <si>
-    <t>precio</t>
-  </si>
-  <si>
-    <t>relacion precio calidad</t>
-  </si>
-  <si>
-    <t>bateria</t>
-  </si>
-  <si>
-    <t>bateria dura mucho</t>
-  </si>
-  <si>
-    <t>camara</t>
-  </si>
-  <si>
-    <t>tiene buena camara</t>
-  </si>
-  <si>
-    <t>memoria</t>
-  </si>
-  <si>
-    <t>tiene buena memoria</t>
-  </si>
-  <si>
-    <t>sonido</t>
-  </si>
-  <si>
-    <t>tiene buen sonido</t>
-  </si>
-  <si>
-    <t>pantalla</t>
-  </si>
-  <si>
-    <t>buena calidad pantalla</t>
-  </si>
-  <si>
-    <t>tamaño</t>
-  </si>
-  <si>
-    <t>tiene buen tamaño</t>
-  </si>
-  <si>
-    <t>sistema</t>
-  </si>
-  <si>
-    <t>sistema operativo bueno</t>
-  </si>
-  <si>
-    <t>diseño</t>
-  </si>
-  <si>
-    <t>celular buen diseño</t>
-  </si>
-  <si>
-    <t>velocidad</t>
-  </si>
-  <si>
-    <t>tiene buena velocidad</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -121,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -445,93 +420,139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cust_needs_three_words</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>relacion precio calidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>bateria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bateria dura mucho</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>memoria</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tiene buena memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>camara</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tiene buena camara</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>sonido</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tiene buen sonido</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>pantalla</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>buena calidad pantalla</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>tamaño</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tiene buen tamaño</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>sistema</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sistema operativo bueno</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>diseño</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>producto lindo diseño</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>velocidad</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>buena velocidad procesamiento</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ultimos cambios tras informe
</commit_message>
<xml_diff>
--- a/data/data_preparation/celulares/df_cust_needs.xlsx
+++ b/data/data_preparation/celulares/df_cust_needs.xlsx
@@ -1,37 +1,112 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E277F7-C9D6-CF40-BCF3-78389FC34947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>cust_needs_three_words</t>
+  </si>
+  <si>
+    <t>precio</t>
+  </si>
+  <si>
+    <t>relacion precio calidad</t>
+  </si>
+  <si>
+    <t>bateria</t>
+  </si>
+  <si>
+    <t>memoria</t>
+  </si>
+  <si>
+    <t>camara</t>
+  </si>
+  <si>
+    <t>sonido</t>
+  </si>
+  <si>
+    <t>pantalla</t>
+  </si>
+  <si>
+    <t>tamaño</t>
+  </si>
+  <si>
+    <t>sistema</t>
+  </si>
+  <si>
+    <t>diseño</t>
+  </si>
+  <si>
+    <t>velocidad</t>
+  </si>
+  <si>
+    <t>batería dure mucho</t>
+  </si>
+  <si>
+    <t>buen sistema operativo</t>
+  </si>
+  <si>
+    <t>saque buenas fotos y videos</t>
+  </si>
+  <si>
+    <t>buena capacidad de almacenamiento</t>
+  </si>
+  <si>
+    <t>buen sonido</t>
+  </si>
+  <si>
+    <t>buena calidad de pantalla</t>
+  </si>
+  <si>
+    <t>tamaño de pantalla grande</t>
+  </si>
+  <si>
+    <t>buena calidad de diseño</t>
+  </si>
+  <si>
+    <t>alta velocidad de procesamiento</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +121,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,139 +445,93 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>cust_needs_three_words</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>precio</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>relacion precio calidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>bateria</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>bateria dura mucho</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>memoria</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>tiene buena memoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>camara</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>tiene buena camara</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>sonido</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>tiene buen sonido</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>pantalla</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>buena calidad pantalla</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>tamaño</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>tiene buen tamaño</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>sistema</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sistema operativo bueno</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>diseño</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>producto lindo diseño</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>velocidad</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>buena velocidad procesamiento</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adapte codigo por cambios de codigo html. Actualice algunas funciones.
</commit_message>
<xml_diff>
--- a/data/data_preparation/celulares/df_cust_needs.xlsx
+++ b/data/data_preparation/celulares/df_cust_needs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBD62D9-A3C5-1745-8E3E-B345CB777967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387F8290-8E4D-D74D-B034-9D676BE6274C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>cust_needs_three_words</t>
   </si>
@@ -28,61 +28,67 @@
     <t>precio</t>
   </si>
   <si>
-    <t>relacion precio calidad</t>
-  </si>
-  <si>
     <t>bateria</t>
   </si>
   <si>
+    <t>camara</t>
+  </si>
+  <si>
     <t>memoria</t>
   </si>
   <si>
-    <t>camara</t>
-  </si>
-  <si>
     <t>sonido</t>
   </si>
   <si>
+    <t>funciones</t>
+  </si>
+  <si>
+    <t>señal</t>
+  </si>
+  <si>
+    <t>tamaño</t>
+  </si>
+  <si>
     <t>pantalla</t>
   </si>
   <si>
-    <t>tamaño</t>
-  </si>
-  <si>
-    <t>sistema</t>
+    <t>velocidad</t>
   </si>
   <si>
     <t>diseño</t>
   </si>
   <si>
-    <t>velocidad</t>
-  </si>
-  <si>
-    <t>capacidad de almacenamiento</t>
-  </si>
-  <si>
-    <t>calidad de fotos y videos</t>
-  </si>
-  <si>
-    <t>calidad de imagen de la pantalla</t>
-  </si>
-  <si>
-    <t>sistema operativo</t>
-  </si>
-  <si>
-    <t>calidad de diseño</t>
-  </si>
-  <si>
-    <t>calidad sonido</t>
-  </si>
-  <si>
-    <t>tamaño de pantalla</t>
-  </si>
-  <si>
-    <t>duracion de la bateria</t>
-  </si>
-  <si>
-    <t>velocidad de procesamiento</t>
+    <t>Relación precio calidad</t>
+  </si>
+  <si>
+    <t>Duración de la batería</t>
+  </si>
+  <si>
+    <t>Calidad de fotos y videos</t>
+  </si>
+  <si>
+    <t>Capacidad de almacenamiento</t>
+  </si>
+  <si>
+    <t>Calidad de sonido</t>
+  </si>
+  <si>
+    <t>Cantidad y calidad de funciones</t>
+  </si>
+  <si>
+    <t>Conectividad</t>
+  </si>
+  <si>
+    <t>Tamaño de pantalla</t>
+  </si>
+  <si>
+    <t>Calidad de imagen de  la pantalla</t>
+  </si>
+  <si>
+    <t>Velocidad de procesamiento</t>
+  </si>
+  <si>
+    <t>Calidad de diseño</t>
   </si>
 </sst>
 </file>
@@ -446,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -459,52 +465,52 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
@@ -512,26 +518,34 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B11" t="s">
-        <v>20</v>
+      <c r="B12" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>